<commit_message>
at chunk step 3
</commit_message>
<xml_diff>
--- a/Documentation/Copilot/Manual Refactoring.xlsx
+++ b/Documentation/Copilot/Manual Refactoring.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MyArduino\Projects\ESP32_Scale\Documentation\Copilot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{770D129D-5051-48DE-97C3-DBD0EF3A76DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FFBC971-0A2C-4904-8F99-EB3DA367F530}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="16080" windowWidth="29040" windowHeight="15840" xr2:uid="{A2DDF546-D711-427A-8885-DE17E2FA6604}"/>
+    <workbookView xWindow="-28920" yWindow="16080" windowWidth="29040" windowHeight="15840" xr2:uid="{A2DDF546-D711-427A-8885-DE17E2FA6604}"/>
   </bookViews>
   <sheets>
     <sheet name="Chunk 1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="15">
   <si>
     <t>baseline compile</t>
   </si>
@@ -532,11 +532,21 @@
       <c r="B3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="5"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
+      <c r="C3" s="5">
+        <v>314843</v>
+      </c>
+      <c r="D3" s="5">
+        <v>21000</v>
+      </c>
+      <c r="E3" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="F3" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
@@ -545,11 +555,21 @@
       <c r="B4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
+      <c r="C4" s="5">
+        <v>314967</v>
+      </c>
+      <c r="D4" s="5">
+        <v>21000</v>
+      </c>
+      <c r="E4" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="F4" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="3">

</xml_diff>

<commit_message>
create scale io module
Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/Documentation/Copilot/Manual Refactoring.xlsx
+++ b/Documentation/Copilot/Manual Refactoring.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MyArduino\Projects\ESP32_Scale\Documentation\Copilot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FFBC971-0A2C-4904-8F99-EB3DA367F530}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0AD0318-AE3C-42C3-91E5-001AF80044EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="16080" windowWidth="29040" windowHeight="15840" xr2:uid="{A2DDF546-D711-427A-8885-DE17E2FA6604}"/>
+    <workbookView xWindow="-120" yWindow="16080" windowWidth="29040" windowHeight="15840" xr2:uid="{A2DDF546-D711-427A-8885-DE17E2FA6604}"/>
   </bookViews>
   <sheets>
     <sheet name="Chunk 1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="15">
   <si>
     <t>baseline compile</t>
   </si>
@@ -471,10 +471,10 @@
   <cols>
     <col min="1" max="1" width="5" style="4" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="29.85546875" style="4" customWidth="1"/>
-    <col min="3" max="3" width="10.7109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.7109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.42578125" style="4" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="11" style="4" bestFit="1" customWidth="1"/>
     <col min="8" max="16384" width="9.140625" style="4"/>
   </cols>
@@ -487,16 +487,16 @@
         <v>5</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>7</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>9</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>10</v>
@@ -509,17 +509,17 @@
       <c r="B2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="5">
+      <c r="C2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="E2" s="5">
         <v>314963</v>
       </c>
-      <c r="D2" s="5">
+      <c r="F2" s="5">
         <v>21000</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F2" s="3" t="b">
-        <v>1</v>
       </c>
       <c r="G2" s="3" t="s">
         <v>14</v>
@@ -532,17 +532,17 @@
       <c r="B3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="5">
+      <c r="C3" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="D3" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="E3" s="5">
         <v>314843</v>
       </c>
-      <c r="D3" s="5">
+      <c r="F3" s="5">
         <v>21000</v>
-      </c>
-      <c r="E3" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="F3" s="3" t="b">
-        <v>1</v>
       </c>
       <c r="G3" s="3" t="s">
         <v>14</v>
@@ -555,17 +555,17 @@
       <c r="B4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C4" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="D4" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="E4" s="5">
         <v>314967</v>
       </c>
-      <c r="D4" s="5">
+      <c r="F4" s="5">
         <v>21000</v>
-      </c>
-      <c r="E4" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="F4" s="3" t="b">
-        <v>1</v>
       </c>
       <c r="G4" s="3" t="s">
         <v>14</v>
@@ -578,11 +578,21 @@
       <c r="B5" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
+      <c r="C5" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="D5" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="E5" s="5">
+        <v>315419</v>
+      </c>
+      <c r="F5" s="5">
+        <v>21000</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
@@ -591,10 +601,10 @@
       <c r="B6" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="5"/>
+      <c r="F6" s="5"/>
       <c r="G6" s="3"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -604,71 +614,71 @@
       <c r="B7" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="5"/>
-      <c r="D7" s="5"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="5"/>
+      <c r="F7" s="5"/>
       <c r="G7" s="3"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C8" s="6"/>
-      <c r="D8" s="6"/>
+      <c r="E8" s="6"/>
+      <c r="F8" s="6"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C9" s="6"/>
-      <c r="D9" s="6"/>
+      <c r="E9" s="6"/>
+      <c r="F9" s="6"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
+      <c r="E10" s="6"/>
+      <c r="F10" s="6"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C11" s="6"/>
-      <c r="D11" s="6"/>
+      <c r="E11" s="6"/>
+      <c r="F11" s="6"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="6"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C13" s="6"/>
-      <c r="D13" s="6"/>
+      <c r="E13" s="6"/>
+      <c r="F13" s="6"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C14" s="6"/>
-      <c r="D14" s="6"/>
+      <c r="E14" s="6"/>
+      <c r="F14" s="6"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C15" s="6"/>
-      <c r="D15" s="6"/>
+      <c r="E15" s="6"/>
+      <c r="F15" s="6"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C16" s="6"/>
-      <c r="D16" s="6"/>
-    </row>
-    <row r="17" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C17" s="6"/>
-      <c r="D17" s="6"/>
-    </row>
-    <row r="18" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C18" s="6"/>
-      <c r="D18" s="6"/>
-    </row>
-    <row r="19" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C19" s="6"/>
-      <c r="D19" s="6"/>
-    </row>
-    <row r="20" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C20" s="6"/>
-      <c r="D20" s="6"/>
-    </row>
-    <row r="21" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C21" s="6"/>
-      <c r="D21" s="6"/>
-    </row>
-    <row r="22" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C22" s="6"/>
-      <c r="D22" s="6"/>
+      <c r="E16" s="6"/>
+      <c r="F16" s="6"/>
+    </row>
+    <row r="17" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E17" s="6"/>
+      <c r="F17" s="6"/>
+    </row>
+    <row r="18" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E18" s="6"/>
+      <c r="F18" s="6"/>
+    </row>
+    <row r="19" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E19" s="6"/>
+      <c r="F19" s="6"/>
+    </row>
+    <row r="20" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E20" s="6"/>
+      <c r="F20" s="6"/>
+    </row>
+    <row r="21" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E21" s="6"/>
+      <c r="F21" s="6"/>
+    </row>
+    <row r="22" spans="5:6" x14ac:dyDescent="0.25">
+      <c r="E22" s="6"/>
+      <c r="F22" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
chunk2 step 1 Create shared input context header
</commit_message>
<xml_diff>
--- a/Documentation/Copilot/Manual Refactoring.xlsx
+++ b/Documentation/Copilot/Manual Refactoring.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MyArduino\Projects\ESP32_Scale\Documentation\Copilot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0AD0318-AE3C-42C3-91E5-001AF80044EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B0E6C2E-AD4F-42E0-ADEB-2BD17B94D5CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="16080" windowWidth="29040" windowHeight="15840" xr2:uid="{A2DDF546-D711-427A-8885-DE17E2FA6604}"/>
+    <workbookView xWindow="28680" yWindow="16080" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{1557E252-C6A5-4BAE-B138-7EC522AF0E5B}"/>
   </bookViews>
   <sheets>
     <sheet name="Chunk 1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="22">
   <si>
     <t>baseline compile</t>
   </si>
@@ -82,6 +82,27 @@
   </si>
   <si>
     <t>PASS</t>
+  </si>
+  <si>
+    <t>Baseline Compile</t>
+  </si>
+  <si>
+    <t>Create shared input context header</t>
+  </si>
+  <si>
+    <t>Extract known weight workflow</t>
+  </si>
+  <si>
+    <t>Extract max propane workflow</t>
+  </si>
+  <si>
+    <t>Extract tank tare workflow</t>
+  </si>
+  <si>
+    <t>Keep loop routing unchanged</t>
+  </si>
+  <si>
+    <t>Serial behavior sanity check</t>
   </si>
 </sst>
 </file>
@@ -132,7 +153,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -152,6 +173,7 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -601,11 +623,21 @@
       <c r="B6" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="5"/>
-      <c r="F6" s="5"/>
-      <c r="G6" s="3"/>
+      <c r="C6" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="D6" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="E6" s="5">
+        <v>315419</v>
+      </c>
+      <c r="F6" s="5">
+        <v>21000</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
@@ -614,11 +646,21 @@
       <c r="B7" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="5"/>
-      <c r="G7" s="3"/>
+      <c r="C7" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="D7" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="E7" s="5">
+        <v>315419</v>
+      </c>
+      <c r="F7" s="5">
+        <v>21000</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E8" s="6"/>
@@ -687,15 +729,15 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{313FA5D5-B3C9-4258-9468-C70F1A7EA1A3}">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="33" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.42578125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -707,20 +749,131 @@
         <v>5</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>7</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>9</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>10</v>
       </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="7">
+        <v>0</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="E2" s="5">
+        <v>315419</v>
+      </c>
+      <c r="F2" s="5">
+        <v>21000</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="7">
+        <v>1</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="D3" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="E3" s="5">
+        <v>315419</v>
+      </c>
+      <c r="F3" s="5">
+        <v>21000</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="7">
+        <v>2</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="7"/>
+      <c r="D4" s="7"/>
+      <c r="E4" s="7"/>
+      <c r="F4" s="7"/>
+      <c r="G4" s="7"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="7">
+        <v>3</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" s="7"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="7"/>
+      <c r="F5" s="7"/>
+      <c r="G5" s="7"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="7">
+        <v>4</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="7"/>
+      <c r="D6" s="7"/>
+      <c r="E6" s="7"/>
+      <c r="F6" s="7"/>
+      <c r="G6" s="7"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="7">
+        <v>5</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" s="7"/>
+      <c r="D7" s="7"/>
+      <c r="E7" s="7"/>
+      <c r="F7" s="7"/>
+      <c r="G7" s="7"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="7">
+        <v>6</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" s="7"/>
+      <c r="D8" s="7"/>
+      <c r="E8" s="7"/>
+      <c r="F8" s="7"/>
+      <c r="G8" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Extract known weight workflow
</commit_message>
<xml_diff>
--- a/Documentation/Copilot/Manual Refactoring.xlsx
+++ b/Documentation/Copilot/Manual Refactoring.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MyArduino\Projects\ESP32_Scale\Documentation\Copilot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B0E6C2E-AD4F-42E0-ADEB-2BD17B94D5CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD341D66-BFCD-4982-AB1C-AC8F7AB5C8AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="16080" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{1557E252-C6A5-4BAE-B138-7EC522AF0E5B}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="22">
   <si>
     <t>baseline compile</t>
   </si>
@@ -817,11 +817,21 @@
       <c r="B4" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
+      <c r="C4" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="D4" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="E4" s="5">
+        <v>315447</v>
+      </c>
+      <c r="F4" s="5">
+        <v>21000</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="7">

</xml_diff>

<commit_message>
Extract max propane workflow
</commit_message>
<xml_diff>
--- a/Documentation/Copilot/Manual Refactoring.xlsx
+++ b/Documentation/Copilot/Manual Refactoring.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MyArduino\Projects\ESP32_Scale\Documentation\Copilot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD341D66-BFCD-4982-AB1C-AC8F7AB5C8AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC934A86-60F1-4F13-933D-40F7E9F9BEA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="16080" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{1557E252-C6A5-4BAE-B138-7EC522AF0E5B}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="22">
   <si>
     <t>baseline compile</t>
   </si>
@@ -840,11 +840,21 @@
       <c r="B5" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
+      <c r="C5" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="D5" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="E5" s="5">
+        <v>315471</v>
+      </c>
+      <c r="F5" s="5">
+        <v>21000</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="7">
@@ -855,8 +865,8 @@
       </c>
       <c r="C6" s="7"/>
       <c r="D6" s="7"/>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
+      <c r="E6" s="5"/>
+      <c r="F6" s="5"/>
       <c r="G6" s="7"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -868,8 +878,8 @@
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
-      <c r="F7" s="7"/>
+      <c r="E7" s="5"/>
+      <c r="F7" s="5"/>
       <c r="G7" s="7"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -881,8 +891,8 @@
       </c>
       <c r="C8" s="7"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
+      <c r="E8" s="5"/>
+      <c r="F8" s="5"/>
       <c r="G8" s="7"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Extract tank tare workflow
</commit_message>
<xml_diff>
--- a/Documentation/Copilot/Manual Refactoring.xlsx
+++ b/Documentation/Copilot/Manual Refactoring.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MyArduino\Projects\ESP32_Scale\Documentation\Copilot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC934A86-60F1-4F13-933D-40F7E9F9BEA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8064FAC2-EE50-4853-B103-4BEF7D3AF402}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="16080" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{1557E252-C6A5-4BAE-B138-7EC522AF0E5B}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="22">
   <si>
     <t>baseline compile</t>
   </si>
@@ -863,11 +863,21 @@
       <c r="B6" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="5"/>
-      <c r="F6" s="5"/>
-      <c r="G6" s="7"/>
+      <c r="C6" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="D6" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="E6" s="5">
+        <v>315499</v>
+      </c>
+      <c r="F6" s="5">
+        <v>21000</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="7">

</xml_diff>

<commit_message>
chunk 2 steps 5 & 6
</commit_message>
<xml_diff>
--- a/Documentation/Copilot/Manual Refactoring.xlsx
+++ b/Documentation/Copilot/Manual Refactoring.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MyArduino\Projects\ESP32_Scale\Documentation\Copilot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8064FAC2-EE50-4853-B103-4BEF7D3AF402}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE2D6407-76CD-402B-9A4C-E3E907F7CDEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="16080" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{1557E252-C6A5-4BAE-B138-7EC522AF0E5B}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="22">
   <si>
     <t>baseline compile</t>
   </si>
@@ -886,11 +886,21 @@
       <c r="B7" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="5"/>
-      <c r="G7" s="7"/>
+      <c r="C7" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="D7" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="E7" s="5">
+        <v>315499</v>
+      </c>
+      <c r="F7" s="5">
+        <v>21000</v>
+      </c>
+      <c r="G7" s="7" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
@@ -899,11 +909,21 @@
       <c r="B8" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="5"/>
-      <c r="F8" s="5"/>
-      <c r="G8" s="7"/>
+      <c r="C8" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="D8" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="E8" s="5">
+        <v>315499</v>
+      </c>
+      <c r="F8" s="5">
+        <v>21000</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>14</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
chunk 3 step 0 base compile
</commit_message>
<xml_diff>
--- a/Documentation/Copilot/Manual Refactoring.xlsx
+++ b/Documentation/Copilot/Manual Refactoring.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MyArduino\Projects\ESP32_Scale\Documentation\Copilot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE2D6407-76CD-402B-9A4C-E3E907F7CDEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DC723CE-9669-4224-B7FB-997EED2715E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="16080" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{1557E252-C6A5-4BAE-B138-7EC522AF0E5B}"/>
+    <workbookView xWindow="28680" yWindow="16080" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{1557E252-C6A5-4BAE-B138-7EC522AF0E5B}"/>
   </bookViews>
   <sheets>
     <sheet name="Chunk 1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="27">
   <si>
     <t>baseline compile</t>
   </si>
@@ -103,6 +103,21 @@
   </si>
   <si>
     <t>Serial behavior sanity check</t>
+  </si>
+  <si>
+    <t>Consolidate workflow type/context declarations</t>
+  </si>
+  <si>
+    <t>Extract level workflow</t>
+  </si>
+  <si>
+    <t>Extract startup tare workflow</t>
+  </si>
+  <si>
+    <t>Extract calibration workflow</t>
+  </si>
+  <si>
+    <t>Cross-workflow command sanity</t>
   </si>
 </sst>
 </file>
@@ -932,8 +947,17 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{272D7D68-E40F-48F1-B7C1-54BE305A510B}">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="44.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
@@ -943,20 +967,108 @@
         <v>5</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>7</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>9</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>10</v>
       </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="7">
+        <v>0</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="E2" s="5">
+        <v>315499</v>
+      </c>
+      <c r="F2" s="5">
+        <v>21000</v>
+      </c>
+      <c r="G2" s="7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="7">
+        <v>1</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="7"/>
+      <c r="G3" s="7"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="7">
+        <v>2</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" s="7"/>
+      <c r="D4" s="7"/>
+      <c r="E4" s="7"/>
+      <c r="F4" s="7"/>
+      <c r="G4" s="7"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="7">
+        <v>3</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" s="7"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="7"/>
+      <c r="F5" s="7"/>
+      <c r="G5" s="7"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="7">
+        <v>4</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" s="7"/>
+      <c r="D6" s="7"/>
+      <c r="E6" s="7"/>
+      <c r="F6" s="7"/>
+      <c r="G6" s="7"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="7">
+        <v>5</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" s="7"/>
+      <c r="D7" s="7"/>
+      <c r="E7" s="7"/>
+      <c r="F7" s="7"/>
+      <c r="G7" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
extract startup tare flow *and fixed lod on startup bug)
</commit_message>
<xml_diff>
--- a/Documentation/Copilot/Manual Refactoring.xlsx
+++ b/Documentation/Copilot/Manual Refactoring.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MyArduino\Projects\ESP32_Scale\Documentation\Copilot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C94C36CE-A70C-4A38-A442-640B3E6DF451}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FCA56B2-AAA6-4D25-8078-8F34A3D60D0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="16080" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{1557E252-C6A5-4BAE-B138-7EC522AF0E5B}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="27">
   <si>
     <t>baseline compile</t>
   </si>
@@ -1058,11 +1058,21 @@
       <c r="B5" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
+      <c r="C5" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="D5" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="E5" s="5">
+        <v>317059</v>
+      </c>
+      <c r="F5" s="5">
+        <v>21000</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="7">

</xml_diff>

<commit_message>
chunk3 step 2.5 extract runtime persistence helper
</commit_message>
<xml_diff>
--- a/Documentation/Copilot/Manual Refactoring.xlsx
+++ b/Documentation/Copilot/Manual Refactoring.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MyArduino\Projects\ESP32_Scale\Documentation\Copilot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FCA56B2-AAA6-4D25-8078-8F34A3D60D0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11606550-7EF7-41DA-BC44-B0CC73B3961B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="16080" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{1557E252-C6A5-4BAE-B138-7EC522AF0E5B}"/>
   </bookViews>
@@ -1065,7 +1065,7 @@
         <v>1</v>
       </c>
       <c r="E5" s="5">
-        <v>317059</v>
+        <v>317055</v>
       </c>
       <c r="F5" s="5">
         <v>21000</v>

</xml_diff>

<commit_message>
chunk3 finished (calibration workflow extracted)
</commit_message>
<xml_diff>
--- a/Documentation/Copilot/Manual Refactoring.xlsx
+++ b/Documentation/Copilot/Manual Refactoring.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MyArduino\Projects\ESP32_Scale\Documentation\Copilot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11606550-7EF7-41DA-BC44-B0CC73B3961B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{425F3AEA-7257-48E2-B455-5C3739189D5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="16080" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{1557E252-C6A5-4BAE-B138-7EC522AF0E5B}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="27">
   <si>
     <t>baseline compile</t>
   </si>
@@ -1081,11 +1081,21 @@
       <c r="B6" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="7"/>
+      <c r="C6" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="D6" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="E6" s="5">
+        <v>317175</v>
+      </c>
+      <c r="F6" s="5">
+        <v>21000</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="7">
@@ -1094,11 +1104,21 @@
       <c r="B7" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
-      <c r="F7" s="7"/>
-      <c r="G7" s="7"/>
+      <c r="C7" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="D7" s="7" t="b">
+        <v>1</v>
+      </c>
+      <c r="E7" s="5">
+        <v>317175</v>
+      </c>
+      <c r="F7" s="5">
+        <v>21000</v>
+      </c>
+      <c r="G7" s="7" t="s">
+        <v>14</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>